<commit_message>
New batch of contacts 2026-10-08-0053
</commit_message>
<xml_diff>
--- a/inbox/new_batch.xlsx
+++ b/inbox/new_batch.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="87">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -1064,6 +1064,9 @@
       <c r="D27" t="s">
         <v>85</v>
       </c>
+      <c r="E27" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
@@ -1078,6 +1081,9 @@
       <c r="D28" t="s">
         <v>85</v>
       </c>
+      <c r="E28" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
@@ -1091,6 +1097,9 @@
       </c>
       <c r="D29" t="s">
         <v>85</v>
+      </c>
+      <c r="E29" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>